<commit_message>
feat: adicionando tabela de triagem no dicionario
</commit_message>
<xml_diff>
--- a/dados/dicionarios/dicionarios.xlsx
+++ b/dados/dicionarios/dicionarios.xlsx
@@ -1092,9 +1092,1273 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C165"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A131" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A132" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A133" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A134" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A135" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A138" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A139" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A140" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A141" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A144" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A164" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A165" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C148"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2799,6 +4063,224 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(500)</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Texto apresentado como pergunta durante a triagem.</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Ordem de exibicao da pergunta.</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>ordem</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>TINYINT(1)</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Indica se a pergunta e uma pergunta raiz (1=sim, 0=nao).</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da resposta de triagem.</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira que referencia a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>fk_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>ENUM('SIM','NAO')</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Resposta possivel para a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a proxima pergunta.</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>fk_proxima_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adicionando tabela de triagem no dicionario (#17)
</commit_message>
<xml_diff>
--- a/dados/dicionarios/dicionarios.xlsx
+++ b/dados/dicionarios/dicionarios.xlsx
@@ -1092,9 +1092,1273 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C165"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A131" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A132" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A133" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A134" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A135" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A138" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A139" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A140" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A141" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A144" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A164" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A165" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C148"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2799,6 +4063,224 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(500)</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Texto apresentado como pergunta durante a triagem.</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Ordem de exibicao da pergunta.</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>ordem</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>TINYINT(1)</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Indica se a pergunta e uma pergunta raiz (1=sim, 0=nao).</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da resposta de triagem.</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira que referencia a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>fk_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>ENUM('SIM','NAO')</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Resposta possivel para a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a proxima pergunta.</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>fk_proxima_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adicionando tabela de triagem no dicionario (#17) (#18)
Co-authored-by: keniti <gustavo.keniti@sptech.school>
</commit_message>
<xml_diff>
--- a/dados/dicionarios/dicionarios.xlsx
+++ b/dados/dicionarios/dicionarios.xlsx
@@ -1092,9 +1092,1273 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C165"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A131" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A132" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A133" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A134" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A135" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A138" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A139" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A140" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A141" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A144" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A164" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A165" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C148"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2799,6 +4063,224 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(500)</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Texto apresentado como pergunta durante a triagem.</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Ordem de exibicao da pergunta.</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>ordem</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>TINYINT(1)</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Indica se a pergunta e uma pergunta raiz (1=sim, 0=nao).</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Tabela triagem_resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>descricao_campo</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Identificador unico da resposta de triagem.</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira que referencia a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>fk_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>ENUM('SIM','NAO')</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Resposta possivel para a pergunta de triagem.</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>resposta</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a proxima pergunta.</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>fk_proxima_pergunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Chave estrangeira opcional que referencia a tabela especialidade.</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>fk_especialidade</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>